<commit_message>
set optimized 'release' build, 30x speedup
</commit_message>
<xml_diff>
--- a/irrgo/doc/mcts-visit-rates.xlsx
+++ b/irrgo/doc/mcts-visit-rates.xlsx
@@ -19,17 +19,33 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t xml:space="preserve">Debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two-minutes</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -89,12 +105,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -221,122 +249,176 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B10:I15"/>
+  <dimension ref="B10:I24"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="1" t="n">
         <f aca="false">D10*E10</f>
         <v>117</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="1" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="1" t="n">
         <f aca="false">E11*F10</f>
         <v>1170</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="n">
+      <c r="B13" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="C13" s="0" t="n">
+      <c r="C13" s="1" t="n">
         <v>166</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>157</v>
       </c>
-      <c r="E13" s="0" t="n">
+      <c r="E13" s="1" t="n">
         <v>174</v>
       </c>
-      <c r="F13" s="1" t="n">
+      <c r="F13" s="2" t="n">
         <f aca="false">AVERAGE(C13:E13)</f>
         <v>165.666666666667</v>
       </c>
-      <c r="G13" s="1" t="n">
+      <c r="G13" s="2" t="n">
         <f aca="false">F13/B13</f>
         <v>3.68148148148148</v>
       </c>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <f aca="false">$F$11/G13</f>
         <v>317.806841046278</v>
       </c>
-      <c r="I13" s="1" t="n">
+      <c r="I13" s="2" t="n">
         <f aca="false">H13/60</f>
         <v>5.29678068410463</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>120</v>
       </c>
-      <c r="C14" s="0" t="n">
+      <c r="C14" s="1" t="n">
         <v>487</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>291</v>
       </c>
-      <c r="E14" s="0" t="n">
+      <c r="E14" s="1" t="n">
         <v>433</v>
       </c>
-      <c r="F14" s="1" t="n">
+      <c r="F14" s="2" t="n">
         <f aca="false">AVERAGE(C14:E14)</f>
         <v>403.666666666667</v>
       </c>
-      <c r="G14" s="1" t="n">
+      <c r="G14" s="2" t="n">
         <f aca="false">F14/B14</f>
         <v>3.36388888888889</v>
       </c>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <f aca="false">$F$11/G14</f>
         <v>347.811725846408</v>
       </c>
-      <c r="I14" s="1" t="n">
+      <c r="I14" s="2" t="n">
         <f aca="false">H14/60</f>
         <v>5.79686209744013</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <f aca="false">5*60</f>
         <v>300</v>
       </c>
-      <c r="C15" s="0" t="n">
+      <c r="C15" s="1" t="n">
         <v>1099</v>
       </c>
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="1" t="n">
         <v>1046</v>
       </c>
-      <c r="E15" s="0" t="n">
+      <c r="E15" s="1" t="n">
         <v>1076</v>
       </c>
-      <c r="F15" s="1" t="n">
+      <c r="F15" s="2" t="n">
         <f aca="false">AVERAGE(C15:E15)</f>
         <v>1073.66666666667</v>
       </c>
-      <c r="G15" s="1" t="n">
+      <c r="G15" s="2" t="n">
         <f aca="false">F15/B15</f>
         <v>3.57888888888889</v>
       </c>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <f aca="false">$F$11/G15</f>
         <v>326.917106488668</v>
       </c>
-      <c r="I15" s="1" t="n">
+      <c r="I15" s="2" t="n">
         <f aca="false">H15/60</f>
         <v>5.4486184414778</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D20" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <f aca="false">F14</f>
+        <v>403.666666666667</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <v>13896</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <f aca="false">E21/D21</f>
+        <v>34.4244426094137</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>3470</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>3415</v>
+      </c>
+      <c r="E24" s="0" t="n">
+        <v>3268</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <f aca="false">AVERAGE(C24:E24)</f>
+        <v>3384.33333333333</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <f aca="false">F24/B24</f>
+        <v>112.811111111111</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <f aca="false">$F$11/G24</f>
+        <v>10.371318822023</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <f aca="false">H24/60</f>
+        <v>0.172855313700384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>